<commit_message>
Remove a stray <p> tag from the A69 NTEE description
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/lookup/bmf_code_lookup.xlsx
+++ b/data/lookup/bmf_code_lookup.xlsx
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4072" uniqueCount="4072">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4073" uniqueCount="4073">
   <si>
     <t>status_code</t>
   </si>
@@ -12250,6 +12250,9 @@
   </si>
   <si>
     <t xml:space="preserve">This is a temporary code for organizations until information is available to classify the entity in major groups A through Y.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Organizations whose primary activity is the operation of a symphony orchestra including youth symphonies.</t>
   </si>
 </sst>
 </file>
@@ -19208,10 +19211,10 @@
         <v>2240</v>
       </c>
       <c r="D34" t="s">
-        <v>3445</v>
+        <v>4072</v>
       </c>
       <c r="E34" t="s">
-        <v>3413</v>
+        <v>3706</v>
       </c>
     </row>
     <row r="35">

</xml_diff>

<commit_message>
Remove a stray <p> tag from the A69 NTEE description (#57)
Co-authored-by: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/lookup/bmf_code_lookup.xlsx
+++ b/data/lookup/bmf_code_lookup.xlsx
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4072" uniqueCount="4072">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4073" uniqueCount="4073">
   <si>
     <t>status_code</t>
   </si>
@@ -12250,6 +12250,9 @@
   </si>
   <si>
     <t xml:space="preserve">This is a temporary code for organizations until information is available to classify the entity in major groups A through Y.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Organizations whose primary activity is the operation of a symphony orchestra including youth symphonies.</t>
   </si>
 </sst>
 </file>
@@ -19208,10 +19211,10 @@
         <v>2240</v>
       </c>
       <c r="D34" t="s">
-        <v>3445</v>
+        <v>4072</v>
       </c>
       <c r="E34" t="s">
-        <v>3413</v>
+        <v>3706</v>
       </c>
     </row>
     <row r="35">

</xml_diff>